<commit_message>
chore(repo): synchronize current project changes
</commit_message>
<xml_diff>
--- a/plan/backlog-freshflow-mvp-12-tuan-updated.xlsx
+++ b/plan/backlog-freshflow-mvp-12-tuan-updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FreshFlow\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F58DFAF0-6A9D-4254-981E-9AC792CA52C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F99A07B0-0871-4FC3-93C8-3FD03B1269E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5840,7 +5840,7 @@
       </c>
       <c r="O7" s="3"/>
       <c r="P7" s="3" t="s">
-        <v>1617</v>
+        <v>33</v>
       </c>
       <c r="Q7" s="3"/>
       <c r="R7" s="3"/>
@@ -5893,7 +5893,7 @@
       </c>
       <c r="O8" s="3"/>
       <c r="P8" s="3" t="s">
-        <v>1617</v>
+        <v>33</v>
       </c>
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="O9" s="3"/>
       <c r="P9" s="3" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
@@ -6005,7 +6005,7 @@
       </c>
       <c r="O10" s="3"/>
       <c r="P10" s="3" t="s">
-        <v>71</v>
+        <v>1617</v>
       </c>
       <c r="Q10" s="3"/>
       <c r="R10" s="3"/>
@@ -15332,7 +15332,7 @@
       </c>
       <c r="B11" s="7" t="str">
         <f>COUNTIF('Backlog 12 Tuan'!P:P,"Done")&amp;" / "&amp;COUNTA('Backlog 12 Tuan'!A:A)-1&amp;" task Done"</f>
-        <v>4 / 168 task Done</v>
+        <v>7 / 168 task Done</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -15341,7 +15341,7 @@
       </c>
       <c r="B12" s="8">
         <f>COUNTIF('Backlog 12 Tuan'!P:P,"Done")/(COUNTA('Backlog 12 Tuan'!A:A)-1)</f>
-        <v>2.3809523809523808E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>